<commit_message>
erd & query SQL - Irza
</commit_message>
<xml_diff>
--- a/Normalisasi_SalesDB_Irza.xlsx
+++ b/Normalisasi_SalesDB_Irza.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fariz Irza\Documents\Magang\Gawe\Database\Latihan-database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD49C5A4-5877-47A5-87CE-9565D0082425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D782C0EF-0490-40E3-9909-3B239F74FC6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Petunjuk" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,8 @@
     <sheet name="2_1NF" sheetId="3" r:id="rId3"/>
     <sheet name="3_2NF" sheetId="4" r:id="rId4"/>
     <sheet name="4_3NF" sheetId="5" r:id="rId5"/>
+    <sheet name="5_ERD" sheetId="6" r:id="rId6"/>
+    <sheet name="6_QuerySQL" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -115,7 +117,7 @@
     <author>Trainer</author>
   </authors>
   <commentList>
-    <comment ref="C13" authorId="0" shapeId="0" xr:uid="{CE614FAC-E9E6-427C-A9FE-51DA32BC456E}">
+    <comment ref="D13" authorId="0" shapeId="0" xr:uid="{CE614FAC-E9E6-427C-A9FE-51DA32BC456E}">
       <text>
         <r>
           <rPr>
@@ -134,7 +136,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="146">
   <si>
     <t>Latihan Normalisasi SalesDB — dari data faktur (UNF) sampai 3NF</t>
   </si>
@@ -595,6 +597,120 @@
   </si>
   <si>
     <t>Menjadi Full semua tabel</t>
+  </si>
+  <si>
+    <t>Kode Kategori (FK)</t>
+  </si>
+  <si>
+    <t>Kode Pelanggan (FK)</t>
+  </si>
+  <si>
+    <t>Tabel Detail_Faktur</t>
+  </si>
+  <si>
+    <t>IF DB_ID(N'SalesDB') IS NULL
+	CREATE DATABASE SalesDB;
+GO
+USE SalesDB
+GO
+CREATE TABLE Costumer (
+CostumerID UNIQUEIDENTIFIER NOT NULL,
+Costumer_Name NVARCHAR(50) NOT NULL,
+Email NVARCHAR(50) NOT NULL,
+City NVARCHAR(50) NOT NULL,
+CONSTRAINT PK_Costumer PRIMARY KEY (CostumerID)
+)
+GO
+CREATE UNIQUE NONCLUSTERED INDEX UQ_Costumer_Email
+	ON dbo.Costumer (Email)
+	WHERE Email IS NOT NULL;
+GO
+CREATE TABLE Category (
+CategoryID INT IDENTITY(1,1) NOT NULL,
+SubCategoryID INT NULL,
+Category_Name NVARCHAR(50) NOT NULL,
+CONSTRAINT PK_Category PRIMARY KEY (CategoryID),
+CONSTRAINT FK_Category_SubCategory FOREIGN KEY (SubCategoryID) REFERENCES Category(CategoryID)
+)
+GO
+CREATE TABLE [Order] (
+OrderID UNIQUEIDENTIFIER NOT NULL,
+CostumerID UNIQUEIDENTIFIER NOT NULL,
+Date DATETIME2 NOT NULL CONSTRAINT DF_Order_Date DEFAULT GETDATE(),
+CONSTRAINT PK_Order PRIMARY KEY (OrderID),
+CONSTRAINT FK_Order_Costumer FOREIGN KEY (CostumerID) REFERENCES Costumer(CostumerID)
+)
+GO
+CREATE TABLE Product (
+ProductID INT IDENTITY(1,1) NOT NULL,
+CategoryID INT NOT NULL,
+Product_Name NVARCHAR(50) NOT NULL,
+Unit_Price DECIMAL(12,2) NOT NULL,
+Stock INT NOT NULL,
+CONSTRAINT PK_Product PRIMARY KEY (ProductID),
+CONSTRAINT FK_Product_Category FOREIGN KEY (CategoryID) REFERENCES Category(CategoryID)
+)
+GO
+CREATE TABLE Order_Detail (
+OrderID UNIQUEIDENTIFIER NOT NULL,
+ProductID INT NOT NULL,
+Quantity INT NOT NULL,
+Unit_Price DECIMAL(12,2) NOT NULL,
+CONSTRAINT PK_Order_Detail PRIMARY KEY (OrderID, ProductID),
+CONSTRAINT FK_Order_Detail_Order FOREIGN KEY (OrderID) REFERENCES [Order](OrderID),
+CONSTRAINT FK_Order_Detail_Product FOREIGN KEY (ProductID) REFERENCES Product(ProductID),
+CONSTRAINT CK_Quantity CHECK (Quantity&gt;0)
+)
+GO
+DECLARE @C1 UNIQUEIDENTIFIER = NEWID();
+DECLARE @C2 UNIQUEIDENTIFIER = NEWID();
+DECLARE @C3 UNIQUEIDENTIFIER = NEWID();
+INSERT INTO dbo.Costumer (CostumerID, Costumer_Name, Email, City)
+VALUES	(@C1, N'Budi Santoso', N'budi@mail.com', 'Jakarta'),
+		(@C2, N'Siti Aminah', N'siti@mail.com', 'Bandung'),
+		(@C3, N'Andi Wijaya', N'andi@mail.com', 'Surabaya');
+INSERT INTO dbo.Category (SubCategoryID, Category_Name)
+VALUES	(NULL, N'Elektronik'),
+		(NULL, N'Alat Tulis'),
+		(NULL, N'Aksesoris Komputer');
+INSERT INTO dbo.Product (CategoryID,	Product_Name, Unit_Price, Stock)
+VALUES	(1, N'Monitor 24 inci', 1850000, 5),
+		(3, N'Headset USB', 350000, 10),
+		(2, N'Buku Catatan A5', 25000, 15),
+		(2, N'Pulpen Gel (isi 12)', 48000, 20),
+		(3, N'Mouse Wireless', 150000, 25),
+		(3, N'Keyboard Mekanik', 750000, 30);
+DECLARE @O1 UNIQUEIDENTIFIER = NEWID();
+DECLARE @O2 UNIQUEIDENTIFIER = NEWID();
+DECLARE @O3 UNIQUEIDENTIFIER = NEWID();
+DECLARE @O4 UNIQUEIDENTIFIER = NEWID();
+DECLARE @O5 UNIQUEIDENTIFIER = NEWID();
+DECLARE @O6 UNIQUEIDENTIFIER = NEWID();
+INSERT INTO dbo.[Order] (OrderID, CostumerID, Date)
+VALUES	(@O1, @C1, '2026-09-01'),
+		(@O2, @C2, '2026-09-10'),
+		(@O3, @C3, '2026-09-12'),
+		(@O4, @C1, '2026-09-15'),
+		(@O5, @C2, '2026-09-18'),
+		(@O6, @C3, '2026-09-20');
+INSERT INTO dbo.Order_Detail (OrderID, ProductID, Quantity, Unit_Price)
+VALUES	(@O1, 1, 1, 1850000),
+		(@O1, 5, 2, 150000),
+		(@O2, 6, 1, 750000),
+		(@O2, 5, 1, 150000),
+		(@O3, 2, 3, 350000),
+		(@O4, 3, 10, 25000),
+		(@O4, 4, 2, 48000),
+		(@O5, 2, 1, 350000),
+		(@O5, 3, 5, 25000),
+		(@O5, 4, 1, 48000),
+		(@O6, 1, 2, 1850000),
+		(@O6, 6, 1, 750000);
+SELECT * FROM Costumer
+SELECT * FROM Category
+SELECT * FROM Product
+SELECT * FROM [Order]
+SELECT * FROM Order_Detail</t>
   </si>
 </sst>
 </file>
@@ -604,7 +720,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mm\-yyyy"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -688,6 +804,18 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF0000FF"/>
+      <name val="Cascadia Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -708,11 +836,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6E0B4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
@@ -725,6 +848,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF8CBAD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6E0B4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -756,7 +885,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -764,7 +893,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -780,7 +908,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -794,19 +922,29 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -816,6 +954,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFC6E0B4"/>
       <color rgb="FFF8CBAD"/>
     </mruColors>
   </colors>
@@ -828,6 +967,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>585305</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>94796</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96C828B4-347D-D60F-2297-2128C5DAFC25}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12777305" cy="6571796"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1222,19 +1410,19 @@
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="7"/>
+      <c r="A24" s="26"/>
       <c r="B24" s="5" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" s="24"/>
+      <c r="A25" s="23"/>
       <c r="B25" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="7" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1263,7 +1451,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1273,322 +1461,322 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="I4" s="19" t="s">
+      <c r="I4" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="J4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="K4" s="10" t="s">
+      <c r="K4" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="L4" s="10" t="s">
+      <c r="L4" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="M4" s="10" t="s">
+      <c r="M4" s="9" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="11">
         <v>46266</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="H5" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="I5" s="20" t="s">
+      <c r="I5" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="J5" s="11" t="s">
+      <c r="J5" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="K5" s="11" t="s">
+      <c r="K5" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="L5" s="11" t="s">
+      <c r="L5" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="M5" s="13">
+      <c r="M5" s="12">
         <v>2150000</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="11">
         <v>46275</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="I6" s="20" t="s">
+      <c r="I6" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="J6" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="K6" s="11" t="s">
+      <c r="K6" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="L6" s="11" t="s">
+      <c r="L6" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="M6" s="13">
+      <c r="M6" s="12">
         <v>900000</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="11">
         <v>46277</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="G7" s="20" t="s">
+      <c r="G7" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="H7" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="I7" s="20" t="s">
+      <c r="I7" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="J7" s="11" t="s">
+      <c r="J7" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="K7" s="11" t="s">
+      <c r="K7" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="L7" s="11" t="s">
+      <c r="L7" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="M7" s="13">
+      <c r="M7" s="12">
         <v>1050000</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="11">
         <v>46280</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="G8" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="I8" s="20" t="s">
+      <c r="I8" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="J8" s="11" t="s">
+      <c r="J8" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="K8" s="11" t="s">
+      <c r="K8" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="L8" s="11" t="s">
+      <c r="L8" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="M8" s="13">
+      <c r="M8" s="12">
         <v>346000</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="11">
         <v>46283</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G9" s="20" t="s">
+      <c r="G9" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="H9" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="I9" s="20" t="s">
+      <c r="I9" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="J9" s="11" t="s">
+      <c r="J9" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="K9" s="11" t="s">
+      <c r="K9" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="L9" s="11" t="s">
+      <c r="L9" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="M9" s="13">
+      <c r="M9" s="12">
         <v>548000</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="11">
         <v>46285</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="H10" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="I10" s="20" t="s">
+      <c r="I10" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="J10" s="11" t="s">
+      <c r="J10" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="K10" s="11" t="s">
+      <c r="K10" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="L10" s="11" t="s">
+      <c r="L10" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="M10" s="13">
+      <c r="M10" s="12">
         <v>4450000</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="17" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="17" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="17" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="17" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="17" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="17" t="s">
         <v>106</v>
       </c>
     </row>
@@ -1619,7 +1807,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>87</v>
       </c>
     </row>
@@ -1639,32 +1827,32 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="15" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="15" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="20" t="s">
         <v>122</v>
       </c>
     </row>
@@ -1674,535 +1862,535 @@
       </c>
     </row>
     <row r="11" spans="1:13" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="H11" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="I11" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="J11" s="10" t="s">
+      <c r="J11" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="K11" s="10" t="s">
+      <c r="K11" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="L11" s="10" t="s">
+      <c r="L11" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="M11" s="10" t="s">
+      <c r="M11" s="9" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="11">
         <v>46266</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="G12" s="22" t="s">
+      <c r="G12" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="H12" s="11" t="s">
+      <c r="H12" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="I12" s="11" t="s">
+      <c r="I12" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="J12" s="11" t="s">
+      <c r="J12" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="K12" s="11">
+      <c r="K12" s="10">
         <v>1</v>
       </c>
-      <c r="L12" s="13">
+      <c r="L12" s="12">
         <v>1850000</v>
       </c>
-      <c r="M12" s="13">
+      <c r="M12" s="12">
         <v>2150000</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="11">
         <v>46266</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="G13" s="22" t="s">
+      <c r="G13" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="H13" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="I13" s="11" t="s">
+      <c r="I13" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="J13" s="11" t="s">
+      <c r="J13" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="K13" s="11">
+      <c r="K13" s="10">
         <v>2</v>
       </c>
-      <c r="L13" s="13">
+      <c r="L13" s="12">
         <v>150000</v>
       </c>
-      <c r="M13" s="13">
+      <c r="M13" s="12">
         <v>2150000</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="11">
         <v>46275</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="F14" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G14" s="22" t="s">
+      <c r="G14" s="21" t="s">
         <v>114</v>
       </c>
-      <c r="H14" s="11" t="s">
+      <c r="H14" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="I14" s="11" t="s">
+      <c r="I14" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="J14" s="11" t="s">
+      <c r="J14" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="K14" s="11">
+      <c r="K14" s="10">
         <v>1</v>
       </c>
-      <c r="L14" s="13">
+      <c r="L14" s="12">
         <v>750000</v>
       </c>
-      <c r="M14" s="13">
+      <c r="M14" s="12">
         <v>900000</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="12">
+      <c r="B15" s="11">
         <v>46275</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G15" s="22" t="s">
+      <c r="G15" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="H15" s="11" t="s">
+      <c r="H15" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="I15" s="11" t="s">
+      <c r="I15" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="J15" s="11" t="s">
+      <c r="J15" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="K15" s="11">
+      <c r="K15" s="10">
         <v>1</v>
       </c>
-      <c r="L15" s="13">
+      <c r="L15" s="12">
         <v>150000</v>
       </c>
-      <c r="M15" s="13">
+      <c r="M15" s="12">
         <v>900000</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="12">
+      <c r="B16" s="11">
         <v>46277</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="F16" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="G16" s="22" t="s">
+      <c r="G16" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="H16" s="11" t="s">
+      <c r="H16" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="I16" s="11" t="s">
+      <c r="I16" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="J16" s="11" t="s">
+      <c r="J16" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="K16" s="11">
+      <c r="K16" s="10">
         <v>3</v>
       </c>
-      <c r="L16" s="13">
+      <c r="L16" s="12">
         <v>350000</v>
       </c>
-      <c r="M16" s="13">
+      <c r="M16" s="12">
         <v>1050000</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="12">
+      <c r="B17" s="11">
         <v>46280</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="F17" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="G17" s="22" t="s">
+      <c r="G17" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="H17" s="11" t="s">
+      <c r="H17" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="I17" s="11" t="s">
+      <c r="I17" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="J17" s="11" t="s">
+      <c r="J17" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="K17" s="11">
+      <c r="K17" s="10">
         <v>10</v>
       </c>
-      <c r="L17" s="13">
+      <c r="L17" s="12">
         <v>25000</v>
       </c>
-      <c r="M17" s="13">
+      <c r="M17" s="12">
         <v>346000</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="B18" s="12">
+      <c r="B18" s="11">
         <v>46280</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="D18" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="E18" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="F18" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="G18" s="22" t="s">
+      <c r="G18" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="H18" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="I18" s="11" t="s">
+      <c r="I18" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="J18" s="11" t="s">
+      <c r="J18" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="K18" s="11">
+      <c r="K18" s="10">
         <v>2</v>
       </c>
-      <c r="L18" s="13">
+      <c r="L18" s="12">
         <v>48000</v>
       </c>
-      <c r="M18" s="13">
+      <c r="M18" s="12">
         <v>346000</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="B19" s="12">
+      <c r="B19" s="11">
         <v>46283</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="E19" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G19" s="22" t="s">
+      <c r="G19" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="H19" s="11" t="s">
+      <c r="H19" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="I19" s="11" t="s">
+      <c r="I19" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="J19" s="11" t="s">
+      <c r="J19" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="K19" s="11">
+      <c r="K19" s="10">
         <v>1</v>
       </c>
-      <c r="L19" s="13">
+      <c r="L19" s="12">
         <v>375000</v>
       </c>
-      <c r="M19" s="13">
+      <c r="M19" s="12">
         <v>548000</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="22" t="s">
+      <c r="A20" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="B20" s="12">
+      <c r="B20" s="11">
         <v>46283</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="F20" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G20" s="22" t="s">
+      <c r="G20" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="H20" s="11" t="s">
+      <c r="H20" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="I20" s="11" t="s">
+      <c r="I20" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="J20" s="11" t="s">
+      <c r="J20" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="K20" s="11">
+      <c r="K20" s="10">
         <v>5</v>
       </c>
-      <c r="L20" s="13">
+      <c r="L20" s="12">
         <v>25000</v>
       </c>
-      <c r="M20" s="13">
+      <c r="M20" s="12">
         <v>548000</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="B21" s="12">
+      <c r="B21" s="11">
         <v>46283</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E21" s="11" t="s">
+      <c r="E21" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="F21" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G21" s="22" t="s">
+      <c r="G21" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="H21" s="11" t="s">
+      <c r="H21" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="I21" s="11" t="s">
+      <c r="I21" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="J21" s="11" t="s">
+      <c r="J21" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="K21" s="11">
+      <c r="K21" s="10">
         <v>1</v>
       </c>
-      <c r="L21" s="13">
+      <c r="L21" s="12">
         <v>48000</v>
       </c>
-      <c r="M21" s="13">
+      <c r="M21" s="12">
         <v>548000</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="B22" s="12">
+      <c r="B22" s="11">
         <v>46285</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="D22" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="E22" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="F22" s="11" t="s">
+      <c r="F22" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="G22" s="22" t="s">
+      <c r="G22" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="H22" s="11" t="s">
+      <c r="H22" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="I22" s="11" t="s">
+      <c r="I22" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="J22" s="11" t="s">
+      <c r="J22" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="K22" s="11">
+      <c r="K22" s="10">
         <v>2</v>
       </c>
-      <c r="L22" s="13">
+      <c r="L22" s="12">
         <v>1850000</v>
       </c>
-      <c r="M22" s="13">
+      <c r="M22" s="12">
         <v>4450000</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="B23" s="12">
+      <c r="B23" s="11">
         <v>46285</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="D23" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E23" s="11" t="s">
+      <c r="E23" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="F23" s="11" t="s">
+      <c r="F23" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="G23" s="22" t="s">
+      <c r="G23" s="21" t="s">
         <v>114</v>
       </c>
-      <c r="H23" s="11" t="s">
+      <c r="H23" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="I23" s="11" t="s">
+      <c r="I23" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="J23" s="11" t="s">
+      <c r="J23" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="K23" s="11">
+      <c r="K23" s="10">
         <v>1</v>
       </c>
-      <c r="L23" s="13">
+      <c r="L23" s="12">
         <v>750000</v>
       </c>
-      <c r="M23" s="13">
+      <c r="M23" s="12">
         <v>4450000</v>
       </c>
     </row>
@@ -2232,7 +2420,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>96</v>
       </c>
     </row>
@@ -2252,28 +2440,28 @@
       </c>
     </row>
     <row r="6" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="C6" s="16"/>
+      <c r="C6" s="15"/>
     </row>
     <row r="7" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="C7" s="16"/>
+      <c r="C7" s="15"/>
     </row>
     <row r="8" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="14" t="s">
         <v>129</v>
       </c>
     </row>
@@ -2288,453 +2476,453 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" s="9" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="11">
         <v>46266</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="G13" s="13">
+      <c r="G13" s="12">
         <v>2150000</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="11">
         <v>46275</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="F14" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G14" s="13">
+      <c r="G14" s="12">
         <v>900000</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="B15" s="12">
+      <c r="B15" s="11">
         <v>46277</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="G15" s="13">
+      <c r="G15" s="12">
         <v>1050000</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="B16" s="12">
+      <c r="B16" s="11">
         <v>46280</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="F16" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="G16" s="13">
+      <c r="G16" s="12">
         <v>346000</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="12">
+      <c r="B17" s="11">
         <v>46283</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="F17" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="G17" s="13">
+      <c r="G17" s="12">
         <v>548000</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="B18" s="12">
+      <c r="B18" s="11">
         <v>46285</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="D18" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="E18" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="F18" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="G18" s="13">
+      <c r="G18" s="12">
         <v>4450000</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="22" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="9" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="D23" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="D24" s="10" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="D25" s="10" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="D26" s="10" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="C27" s="11" t="s">
+      <c r="C27" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="D27" s="11" t="s">
+      <c r="D27" s="10" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="22" t="s">
+      <c r="A28" s="21" t="s">
         <v>114</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="D28" s="11" t="s">
+      <c r="D28" s="10" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="23" t="s">
+      <c r="A31" s="22" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="19" t="s">
+      <c r="A32" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B32" s="19" t="s">
+      <c r="B32" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="10" t="s">
+      <c r="D32" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="25" t="s">
+      <c r="A33" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="25" t="s">
+      <c r="B33" s="24" t="s">
         <v>107</v>
       </c>
-      <c r="C33" s="11">
+      <c r="C33" s="10">
         <v>1</v>
       </c>
-      <c r="D33" s="13">
+      <c r="D33" s="12">
         <v>1850000</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="25" t="s">
+      <c r="A34" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="B34" s="25" t="s">
+      <c r="B34" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="C34" s="11">
+      <c r="C34" s="10">
         <v>2</v>
       </c>
-      <c r="D34" s="13">
+      <c r="D34" s="12">
         <v>150000</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="25" t="s">
+      <c r="A35" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="B35" s="25" t="s">
+      <c r="B35" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="C35" s="11">
+      <c r="C35" s="10">
         <v>1</v>
       </c>
-      <c r="D35" s="13">
+      <c r="D35" s="12">
         <v>750000</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="25" t="s">
+      <c r="A36" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="B36" s="25" t="s">
+      <c r="B36" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="C36" s="11">
+      <c r="C36" s="10">
         <v>1</v>
       </c>
-      <c r="D36" s="13">
+      <c r="D36" s="12">
         <v>150000</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="25" t="s">
+      <c r="A37" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="B37" s="25" t="s">
+      <c r="B37" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="C37" s="11">
+      <c r="C37" s="10">
         <v>3</v>
       </c>
-      <c r="D37" s="13">
+      <c r="D37" s="12">
         <v>350000</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="25" t="s">
+      <c r="A38" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="B38" s="25" t="s">
+      <c r="B38" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="C38" s="11">
+      <c r="C38" s="10">
         <v>10</v>
       </c>
-      <c r="D38" s="13">
+      <c r="D38" s="12">
         <v>25000</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39" s="25" t="s">
+      <c r="A39" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="B39" s="25" t="s">
+      <c r="B39" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="C39" s="11">
+      <c r="C39" s="10">
         <v>2</v>
       </c>
-      <c r="D39" s="13">
+      <c r="D39" s="12">
         <v>48000</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="25" t="s">
+      <c r="A40" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="B40" s="25" t="s">
+      <c r="B40" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="C40" s="11">
+      <c r="C40" s="10">
         <v>1</v>
       </c>
-      <c r="D40" s="13">
+      <c r="D40" s="12">
         <v>350000</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="25" t="s">
+      <c r="A41" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="B41" s="25" t="s">
+      <c r="B41" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="C41" s="11">
+      <c r="C41" s="10">
         <v>5</v>
       </c>
-      <c r="D41" s="13">
+      <c r="D41" s="12">
         <v>25000</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" s="25" t="s">
+      <c r="A42" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="B42" s="25" t="s">
+      <c r="B42" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="C42" s="11">
+      <c r="C42" s="10">
         <v>1</v>
       </c>
-      <c r="D42" s="13">
+      <c r="D42" s="12">
         <v>48000</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43" s="25" t="s">
+      <c r="A43" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B43" s="25" t="s">
+      <c r="B43" s="24" t="s">
         <v>107</v>
       </c>
-      <c r="C43" s="11">
+      <c r="C43" s="10">
         <v>2</v>
       </c>
-      <c r="D43" s="13">
+      <c r="D43" s="12">
         <v>1850000</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" s="25" t="s">
+      <c r="A44" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B44" s="25" t="s">
+      <c r="B44" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="C44" s="11">
+      <c r="C44" s="10">
         <v>1</v>
       </c>
-      <c r="D44" s="13">
+      <c r="D44" s="12">
         <v>750000</v>
       </c>
     </row>
@@ -2752,489 +2940,531 @@
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="17.77734375" customWidth="1"/>
+    <col min="4" max="4" width="26.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
+    <row r="6" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="15" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
+    <row r="7" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="15" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
+    <row r="8" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="14" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="19" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="22" t="s">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="11">
         <v>46266</v>
       </c>
-      <c r="C13" s="13">
+      <c r="C13" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="12">
         <v>2150000</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="22" t="s">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="11">
         <v>46275</v>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="27" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="12">
         <v>900000</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="22" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="B15" s="12">
+      <c r="B15" s="11">
         <v>46277</v>
       </c>
-      <c r="C15" s="13">
+      <c r="C15" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="12">
         <v>1050000</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="22" t="s">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="B16" s="12">
+      <c r="B16" s="11">
         <v>46280</v>
       </c>
-      <c r="C16" s="13">
+      <c r="C16" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="12">
         <v>346000</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="12">
+      <c r="B17" s="11">
         <v>46283</v>
       </c>
-      <c r="C17" s="13">
+      <c r="C17" s="27" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="12">
         <v>548000</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="B18" s="12">
+      <c r="B18" s="11">
         <v>46285</v>
       </c>
-      <c r="C18" s="13">
+      <c r="C18" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="12">
         <v>4450000</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="22" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="9" t="s">
         <v>29</v>
       </c>
+      <c r="C22" s="18" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="10" t="s">
         <v>109</v>
       </c>
+      <c r="C23" s="27" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="10" t="s">
         <v>63</v>
       </c>
+      <c r="C24" s="27" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="10" t="s">
         <v>119</v>
       </c>
+      <c r="C25" s="27" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="10" t="s">
         <v>116</v>
       </c>
+      <c r="C26" s="27" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="10" t="s">
         <v>110</v>
       </c>
+      <c r="C27" s="27" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="22" t="s">
+      <c r="A28" s="21" t="s">
         <v>114</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="10" t="s">
         <v>113</v>
       </c>
+      <c r="C28" s="27" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="23" t="s">
-        <v>127</v>
+      <c r="A31" s="22" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="19" t="s">
+      <c r="A32" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="B32" s="19" t="s">
+      <c r="B32" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="10" t="s">
+      <c r="D32" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="25" t="s">
+      <c r="A33" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="25" t="s">
+      <c r="B33" s="24" t="s">
         <v>107</v>
       </c>
-      <c r="C33" s="11">
+      <c r="C33" s="10">
         <v>1</v>
       </c>
-      <c r="D33" s="13">
+      <c r="D33" s="12">
         <v>1850000</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="25" t="s">
+      <c r="A34" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="B34" s="25" t="s">
+      <c r="B34" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="C34" s="11">
+      <c r="C34" s="10">
         <v>2</v>
       </c>
-      <c r="D34" s="13">
+      <c r="D34" s="12">
         <v>150000</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="25" t="s">
+      <c r="A35" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="B35" s="25" t="s">
+      <c r="B35" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="C35" s="11">
+      <c r="C35" s="10">
         <v>1</v>
       </c>
-      <c r="D35" s="13">
+      <c r="D35" s="12">
         <v>750000</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="25" t="s">
+      <c r="A36" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="B36" s="25" t="s">
+      <c r="B36" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="C36" s="11">
+      <c r="C36" s="10">
         <v>1</v>
       </c>
-      <c r="D36" s="13">
+      <c r="D36" s="12">
         <v>150000</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="25" t="s">
+      <c r="A37" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="B37" s="25" t="s">
+      <c r="B37" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="C37" s="11">
+      <c r="C37" s="10">
         <v>3</v>
       </c>
-      <c r="D37" s="13">
+      <c r="D37" s="12">
         <v>350000</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="25" t="s">
+      <c r="A38" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="B38" s="25" t="s">
+      <c r="B38" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="C38" s="11">
+      <c r="C38" s="10">
         <v>10</v>
       </c>
-      <c r="D38" s="13">
+      <c r="D38" s="12">
         <v>25000</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39" s="25" t="s">
+      <c r="A39" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="B39" s="25" t="s">
+      <c r="B39" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="C39" s="11">
+      <c r="C39" s="10">
         <v>2</v>
       </c>
-      <c r="D39" s="13">
+      <c r="D39" s="12">
         <v>48000</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="25" t="s">
+      <c r="A40" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="B40" s="25" t="s">
+      <c r="B40" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="C40" s="11">
+      <c r="C40" s="10">
         <v>1</v>
       </c>
-      <c r="D40" s="13">
+      <c r="D40" s="12">
         <v>350000</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="25" t="s">
+      <c r="A41" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="B41" s="25" t="s">
+      <c r="B41" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="C41" s="11">
+      <c r="C41" s="10">
         <v>5</v>
       </c>
-      <c r="D41" s="13">
+      <c r="D41" s="12">
         <v>25000</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" s="25" t="s">
+      <c r="A42" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="B42" s="25" t="s">
+      <c r="B42" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="C42" s="11">
+      <c r="C42" s="10">
         <v>1</v>
       </c>
-      <c r="D42" s="13">
+      <c r="D42" s="12">
         <v>48000</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43" s="25" t="s">
+      <c r="A43" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B43" s="25" t="s">
+      <c r="B43" s="24" t="s">
         <v>107</v>
       </c>
-      <c r="C43" s="11">
+      <c r="C43" s="10">
         <v>2</v>
       </c>
-      <c r="D43" s="13">
+      <c r="D43" s="12">
         <v>1850000</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" s="25" t="s">
+      <c r="A44" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B44" s="25" t="s">
+      <c r="B44" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="C44" s="11">
+      <c r="C44" s="10">
         <v>1</v>
       </c>
-      <c r="D44" s="13">
+      <c r="D44" s="12">
         <v>750000</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A47" s="26" t="s">
+      <c r="A47" s="25" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A48" s="19" t="s">
+      <c r="A48" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="B48" s="10" t="s">
+      <c r="B48" s="9" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="22" t="s">
+      <c r="A49" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="B49" s="11" t="s">
+      <c r="B49" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A50" s="22" t="s">
+      <c r="A50" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="B50" s="11" t="s">
+      <c r="B50" s="10" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A51" s="22" t="s">
+      <c r="A51" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="B51" s="11" t="s">
+      <c r="B51" s="10" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A54" s="23" t="s">
+      <c r="A54" s="22" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A55" s="19" t="s">
+      <c r="A55" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="B55" s="10" t="s">
+      <c r="B55" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C55" s="10" t="s">
+      <c r="C55" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D55" s="10" t="s">
+      <c r="D55" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A56" s="22" t="s">
+      <c r="A56" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="B56" s="11" t="s">
+      <c r="B56" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C56" s="11" t="s">
+      <c r="C56" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="D56" s="11" t="s">
+      <c r="D56" s="10" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A57" s="22" t="s">
+      <c r="A57" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="B57" s="11" t="s">
+      <c r="B57" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C57" s="11" t="s">
+      <c r="C57" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D57" s="11" t="s">
+      <c r="D57" s="10" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A58" s="22" t="s">
+      <c r="A58" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="B58" s="11" t="s">
+      <c r="B58" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C58" s="11" t="s">
+      <c r="C58" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="D58" s="11" t="s">
+      <c r="D58" s="10" t="s">
         <v>61</v>
       </c>
     </row>
@@ -3242,4 +3472,387 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{789E4B3C-B193-45E4-A791-FA15540AE0B3}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53738DD1-9626-4D9D-9745-E58F6C13D459}">
+  <dimension ref="A1:A118"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="95.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="28" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="29"/>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="29"/>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="29"/>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="29"/>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="29"/>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="29"/>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" s="29"/>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" s="29"/>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" s="29"/>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" s="29"/>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" s="29"/>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" s="29"/>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" s="29"/>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A15" s="29"/>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" s="29"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="29"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="29"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" s="29"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" s="29"/>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" s="29"/>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" s="29"/>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" s="29"/>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" s="29"/>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" s="29"/>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" s="29"/>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" s="29"/>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28" s="29"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" s="29"/>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30" s="29"/>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31" s="29"/>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A32" s="29"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" s="29"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" s="29"/>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" s="29"/>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36" s="29"/>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A37" s="29"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38" s="29"/>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A39" s="29"/>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A40" s="29"/>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A41" s="29"/>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A42" s="29"/>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A43" s="29"/>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A44" s="29"/>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A45" s="29"/>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A46" s="29"/>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A47" s="29"/>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A48" s="29"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" s="29"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" s="29"/>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51" s="29"/>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52" s="29"/>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A53" s="29"/>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A54" s="29"/>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A55" s="29"/>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56" s="29"/>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A57" s="29"/>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A58" s="29"/>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A59" s="29"/>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A60" s="29"/>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A61" s="29"/>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A62" s="29"/>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A63" s="29"/>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A64" s="29"/>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A65" s="29"/>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A66" s="29"/>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A67" s="29"/>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A68" s="29"/>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A69" s="29"/>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A70" s="29"/>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A71" s="29"/>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A72" s="29"/>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A73" s="29"/>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A74" s="29"/>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A75" s="29"/>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A76" s="29"/>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A77" s="29"/>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A78" s="29"/>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A79" s="29"/>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A80" s="29"/>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A81" s="29"/>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A82" s="29"/>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A83" s="29"/>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A84" s="29"/>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A85" s="29"/>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A86" s="29"/>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A87" s="29"/>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A88" s="29"/>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A89" s="29"/>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A90" s="29"/>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A91" s="29"/>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A92" s="29"/>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A93" s="29"/>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A94" s="29"/>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A95" s="29"/>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A96" s="29"/>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A97" s="29"/>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A98" s="29"/>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A99" s="29"/>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A100" s="29"/>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A101" s="29"/>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A102" s="29"/>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A103" s="29"/>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A104" s="29"/>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A105" s="29"/>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A106" s="29"/>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A107" s="29"/>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A108" s="29"/>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A109" s="29"/>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A110" s="29"/>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A111" s="29"/>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A112" s="29"/>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A113" s="29"/>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A114" s="29"/>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A115" s="29"/>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A116" s="29"/>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A117" s="29"/>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A118" s="29"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:A118"/>
+  </mergeCells>
+  <phoneticPr fontId="14" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>